<commit_message>
risultati prima parte dataset 1 e 2
</commit_message>
<xml_diff>
--- a/Results_metrics.xlsx
+++ b/Results_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Enrica\Desktop\Nuovo_ML_Project\MaskArchitectureAnomaly_CourseProject\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gaiac\Desktop\polito\machine learning\MaskArchitectureAnomaly_CourseProject\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1523F03-0172-4C2F-A11F-EE0114E63202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E140A3-96B4-4D03-8875-7623017B2363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11232" yWindow="0" windowWidth="11808" windowHeight="12072" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="51">
   <si>
     <t>Model</t>
   </si>
@@ -172,6 +172,12 @@
   </si>
   <si>
     <t>RISULTATI METRICHE per EoMT con TEMPERATURE su MSP con Logitnorm tau = 0,10</t>
+  </si>
+  <si>
+    <t>81.7%</t>
+  </si>
+  <si>
+    <t>t = 0,2</t>
   </si>
 </sst>
 </file>
@@ -721,10 +727,16 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -750,12 +762,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -901,7 +907,7 @@
                   <c:v>t = 0,1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>t = 0,25</c:v>
+                  <c:v>t = 0,2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>t = 0,5</c:v>
@@ -970,67 +976,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>34.29</c:v>
+                  <c:v>74.77</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>42.38</c:v>
+                  <c:v>74.209999999999994</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>54.02</c:v>
+                  <c:v>73.64</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>58.57</c:v>
+                  <c:v>73.27</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>61.18</c:v>
+                  <c:v>72.95</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>63.4</c:v>
+                  <c:v>73.849999999999994</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>64.28</c:v>
+                  <c:v>74.3</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>65.13</c:v>
+                  <c:v>74.650000000000006</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>67.64</c:v>
+                  <c:v>75.36</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>75.12</c:v>
+                  <c:v>79.150000000000006</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>79.900000000000006</c:v>
+                  <c:v>83.99</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>82.66</c:v>
+                  <c:v>84.35</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>83.9</c:v>
+                  <c:v>84.2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>84.85</c:v>
+                  <c:v>83.5</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>85.12</c:v>
+                  <c:v>82.83</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>85.25</c:v>
+                  <c:v>82.29</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>85.33</c:v>
+                  <c:v>81.849999999999994</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>85.38</c:v>
+                  <c:v>81.5</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>85.42</c:v>
+                  <c:v>81.2</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>85.45</c:v>
+                  <c:v>80.95</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>85.47</c:v>
+                  <c:v>80.7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1089,7 +1095,7 @@
                   <c:v>t = 0,1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>t = 0,25</c:v>
+                  <c:v>t = 0,2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>t = 0,5</c:v>
@@ -1158,67 +1164,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>91.9</c:v>
+                  <c:v>52.9</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>89.39</c:v>
+                  <c:v>52.9</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>30.4</c:v>
+                  <c:v>53.37</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>28.71</c:v>
+                  <c:v>47.2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>28.38</c:v>
+                  <c:v>47.26</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>27.09</c:v>
+                  <c:v>33.659999999999997</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>26.47</c:v>
+                  <c:v>29.93</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>25.89</c:v>
+                  <c:v>27.46</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>24.34</c:v>
+                  <c:v>23.22</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>9.82</c:v>
+                  <c:v>11.57</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>6.72</c:v>
+                  <c:v>4.24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>4.93</c:v>
+                  <c:v>3.64</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.91</c:v>
+                  <c:v>3.52</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.18</c:v>
+                  <c:v>3.6</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2.97</c:v>
+                  <c:v>3.73</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2.86</c:v>
+                  <c:v>3.84</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>2.8</c:v>
+                  <c:v>3.93</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2.76</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>2.73</c:v>
+                  <c:v>4.07</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2.7</c:v>
+                  <c:v>4.12</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.68</c:v>
+                  <c:v>4.1900000000000004</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1670,7 +1676,7 @@
                   <c:v>t = 0,1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>t = 0,25</c:v>
+                  <c:v>t = 0,2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>t = 0,5</c:v>
@@ -1739,67 +1745,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>33.64</c:v>
+                  <c:v>79.37</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>60.22</c:v>
+                  <c:v>81.89</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>75.39</c:v>
+                  <c:v>88.05</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>78.2</c:v>
+                  <c:v>89.79</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>78.75</c:v>
+                  <c:v>89.9</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>80.95</c:v>
+                  <c:v>90.08</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>82</c:v>
+                  <c:v>89.98</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>82.96</c:v>
+                  <c:v>89.67</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>85.28</c:v>
+                  <c:v>84.83</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>88.12</c:v>
+                  <c:v>72.66</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>90.94</c:v>
+                  <c:v>63.45</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>91</c:v>
+                  <c:v>56.31</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>91.17</c:v>
+                  <c:v>51.7</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>91.29</c:v>
+                  <c:v>45.62</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>91.31</c:v>
+                  <c:v>42.33</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>91.31</c:v>
+                  <c:v>39.26</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>91.31</c:v>
+                  <c:v>37.42</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>91.3</c:v>
+                  <c:v>36.72</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>91.3</c:v>
+                  <c:v>36.28</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>91.3</c:v>
+                  <c:v>35.979999999999997</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>91.29</c:v>
+                  <c:v>35.75</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1858,7 +1864,7 @@
                   <c:v>t = 0,1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>t = 0,25</c:v>
+                  <c:v>t = 0,2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>t = 0,5</c:v>
@@ -1927,67 +1933,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>91.83</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>82.2</c:v>
+                  <c:v>2.16</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>26.43</c:v>
+                  <c:v>0.61</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>17.52</c:v>
+                  <c:v>0.54</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>16.989999999999998</c:v>
+                  <c:v>0.54</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>14.95</c:v>
+                  <c:v>0.57999999999999996</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>14.28</c:v>
+                  <c:v>0.62</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>10.92</c:v>
+                  <c:v>0.68</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>11.74</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>12.57</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>15.04</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>16.91</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>17.68</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>19.440000000000001</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>20.47</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>21.04</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>21.37</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>21.52</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>21.62</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>21.75</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>21.84</c:v>
+                  <c:v>100</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2439,7 +2445,7 @@
                   <c:v>t = 0,1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>t = 0,25</c:v>
+                  <c:v>t = 0,2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>t = 0,5</c:v>
@@ -2627,7 +2633,7 @@
                   <c:v>t = 0,1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>t = 0,25</c:v>
+                  <c:v>t = 0,2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>t = 0,5</c:v>
@@ -3208,7 +3214,7 @@
                   <c:v>t = 0,1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>t = 0,25</c:v>
+                  <c:v>t = 0,2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>t = 0,5</c:v>
@@ -3396,7 +3402,7 @@
                   <c:v>t = 0,1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>t = 0,25</c:v>
+                  <c:v>t = 0,2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>t = 0,5</c:v>
@@ -3977,7 +3983,7 @@
                   <c:v>t = 0,1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>t = 0,25</c:v>
+                  <c:v>t = 0,2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>t = 0,5</c:v>
@@ -4147,7 +4153,7 @@
                   <c:v>t = 0,1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>t = 0,25</c:v>
+                  <c:v>t = 0,2</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>t = 0,5</c:v>
@@ -7755,198 +7761,198 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:CB38"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="14.44140625" customWidth="1"/>
-    <col min="3" max="3" width="13.109375" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="45" t="s">
+    <row r="1" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="2" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B2" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
-      <c r="G2" s="50"/>
-      <c r="H2" s="50"/>
-      <c r="I2" s="50"/>
-      <c r="J2" s="50"/>
-      <c r="K2" s="50"/>
-      <c r="L2" s="50"/>
-      <c r="M2" s="51"/>
-      <c r="AA2" s="45" t="s">
+      <c r="C2" s="52"/>
+      <c r="D2" s="52"/>
+      <c r="E2" s="52"/>
+      <c r="F2" s="52"/>
+      <c r="G2" s="52"/>
+      <c r="H2" s="52"/>
+      <c r="I2" s="52"/>
+      <c r="J2" s="52"/>
+      <c r="K2" s="52"/>
+      <c r="L2" s="52"/>
+      <c r="M2" s="53"/>
+      <c r="AA2" s="47" t="s">
         <v>41</v>
       </c>
-      <c r="AB2" s="50"/>
-      <c r="AC2" s="50"/>
-      <c r="AD2" s="50"/>
-      <c r="AE2" s="50"/>
-      <c r="AF2" s="50"/>
-      <c r="AG2" s="50"/>
-      <c r="AH2" s="50"/>
-      <c r="AI2" s="50"/>
-      <c r="AJ2" s="50"/>
-      <c r="AK2" s="50"/>
-      <c r="AL2" s="51"/>
-      <c r="AO2" s="45" t="s">
+      <c r="AB2" s="52"/>
+      <c r="AC2" s="52"/>
+      <c r="AD2" s="52"/>
+      <c r="AE2" s="52"/>
+      <c r="AF2" s="52"/>
+      <c r="AG2" s="52"/>
+      <c r="AH2" s="52"/>
+      <c r="AI2" s="52"/>
+      <c r="AJ2" s="52"/>
+      <c r="AK2" s="52"/>
+      <c r="AL2" s="53"/>
+      <c r="AO2" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="AP2" s="50"/>
-      <c r="AQ2" s="50"/>
-      <c r="AR2" s="50"/>
-      <c r="AS2" s="50"/>
-      <c r="AT2" s="50"/>
-      <c r="AU2" s="50"/>
-      <c r="AV2" s="50"/>
-      <c r="AW2" s="50"/>
-      <c r="AX2" s="50"/>
-      <c r="AY2" s="50"/>
-      <c r="AZ2" s="51"/>
-      <c r="BC2" s="45" t="s">
+      <c r="AP2" s="52"/>
+      <c r="AQ2" s="52"/>
+      <c r="AR2" s="52"/>
+      <c r="AS2" s="52"/>
+      <c r="AT2" s="52"/>
+      <c r="AU2" s="52"/>
+      <c r="AV2" s="52"/>
+      <c r="AW2" s="52"/>
+      <c r="AX2" s="52"/>
+      <c r="AY2" s="52"/>
+      <c r="AZ2" s="53"/>
+      <c r="BC2" s="47" t="s">
         <v>45</v>
       </c>
-      <c r="BD2" s="50"/>
-      <c r="BE2" s="50"/>
-      <c r="BF2" s="50"/>
-      <c r="BG2" s="50"/>
-      <c r="BH2" s="50"/>
-      <c r="BI2" s="50"/>
-      <c r="BJ2" s="50"/>
-      <c r="BK2" s="50"/>
-      <c r="BL2" s="50"/>
-      <c r="BM2" s="50"/>
-      <c r="BN2" s="51"/>
-      <c r="BQ2" s="45" t="s">
+      <c r="BD2" s="52"/>
+      <c r="BE2" s="52"/>
+      <c r="BF2" s="52"/>
+      <c r="BG2" s="52"/>
+      <c r="BH2" s="52"/>
+      <c r="BI2" s="52"/>
+      <c r="BJ2" s="52"/>
+      <c r="BK2" s="52"/>
+      <c r="BL2" s="52"/>
+      <c r="BM2" s="52"/>
+      <c r="BN2" s="53"/>
+      <c r="BQ2" s="47" t="s">
         <v>47</v>
       </c>
-      <c r="BR2" s="50"/>
-      <c r="BS2" s="50"/>
-      <c r="BT2" s="50"/>
-      <c r="BU2" s="50"/>
-      <c r="BV2" s="50"/>
-      <c r="BW2" s="50"/>
-      <c r="BX2" s="50"/>
-      <c r="BY2" s="50"/>
-      <c r="BZ2" s="50"/>
-      <c r="CA2" s="50"/>
-      <c r="CB2" s="51"/>
+      <c r="BR2" s="52"/>
+      <c r="BS2" s="52"/>
+      <c r="BT2" s="52"/>
+      <c r="BU2" s="52"/>
+      <c r="BV2" s="52"/>
+      <c r="BW2" s="52"/>
+      <c r="BX2" s="52"/>
+      <c r="BY2" s="52"/>
+      <c r="BZ2" s="52"/>
+      <c r="CA2" s="52"/>
+      <c r="CB2" s="53"/>
     </row>
-    <row r="3" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B3" s="1"/>
       <c r="C3" s="5"/>
-      <c r="D3" s="48" t="s">
+      <c r="D3" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="E3" s="49"/>
-      <c r="F3" s="48" t="s">
+      <c r="E3" s="51"/>
+      <c r="F3" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="49"/>
-      <c r="H3" s="48" t="s">
+      <c r="G3" s="51"/>
+      <c r="H3" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="I3" s="49"/>
-      <c r="J3" s="48" t="s">
+      <c r="I3" s="51"/>
+      <c r="J3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="49"/>
-      <c r="L3" s="48" t="s">
+      <c r="K3" s="51"/>
+      <c r="L3" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="M3" s="49"/>
+      <c r="M3" s="51"/>
       <c r="AA3" s="1"/>
       <c r="AB3" s="5"/>
-      <c r="AC3" s="48" t="s">
+      <c r="AC3" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="AD3" s="49"/>
-      <c r="AE3" s="48" t="s">
+      <c r="AD3" s="51"/>
+      <c r="AE3" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="AF3" s="49"/>
-      <c r="AG3" s="48" t="s">
+      <c r="AF3" s="51"/>
+      <c r="AG3" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="AH3" s="49"/>
-      <c r="AI3" s="48" t="s">
+      <c r="AH3" s="51"/>
+      <c r="AI3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="AJ3" s="49"/>
-      <c r="AK3" s="48" t="s">
+      <c r="AJ3" s="51"/>
+      <c r="AK3" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="AL3" s="49"/>
+      <c r="AL3" s="51"/>
       <c r="AO3" s="1"/>
       <c r="AP3" s="5"/>
-      <c r="AQ3" s="48" t="s">
+      <c r="AQ3" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="AR3" s="49"/>
-      <c r="AS3" s="48" t="s">
+      <c r="AR3" s="51"/>
+      <c r="AS3" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="AT3" s="49"/>
-      <c r="AU3" s="48" t="s">
+      <c r="AT3" s="51"/>
+      <c r="AU3" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="AV3" s="49"/>
-      <c r="AW3" s="48" t="s">
+      <c r="AV3" s="51"/>
+      <c r="AW3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="AX3" s="49"/>
-      <c r="AY3" s="48" t="s">
+      <c r="AX3" s="51"/>
+      <c r="AY3" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="AZ3" s="49"/>
+      <c r="AZ3" s="51"/>
       <c r="BC3" s="1"/>
       <c r="BD3" s="5"/>
-      <c r="BE3" s="48" t="s">
+      <c r="BE3" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="BF3" s="49"/>
-      <c r="BG3" s="48" t="s">
+      <c r="BF3" s="51"/>
+      <c r="BG3" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="BH3" s="49"/>
-      <c r="BI3" s="48" t="s">
+      <c r="BH3" s="51"/>
+      <c r="BI3" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="BJ3" s="49"/>
-      <c r="BK3" s="48" t="s">
+      <c r="BJ3" s="51"/>
+      <c r="BK3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="BL3" s="49"/>
-      <c r="BM3" s="48" t="s">
+      <c r="BL3" s="51"/>
+      <c r="BM3" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="BN3" s="49"/>
+      <c r="BN3" s="51"/>
       <c r="BQ3" s="1"/>
       <c r="BR3" s="5"/>
-      <c r="BS3" s="48" t="s">
+      <c r="BS3" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="BT3" s="49"/>
-      <c r="BU3" s="48" t="s">
+      <c r="BT3" s="51"/>
+      <c r="BU3" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="BV3" s="49"/>
-      <c r="BW3" s="48" t="s">
+      <c r="BV3" s="51"/>
+      <c r="BW3" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="BX3" s="49"/>
-      <c r="BY3" s="48" t="s">
+      <c r="BX3" s="51"/>
+      <c r="BY3" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="BZ3" s="49"/>
-      <c r="CA3" s="48" t="s">
+      <c r="BZ3" s="51"/>
+      <c r="CA3" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="CB3" s="49"/>
+      <c r="CB3" s="51"/>
     </row>
-    <row r="4" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="6" t="s">
         <v>0</v>
       </c>
@@ -8128,8 +8134,8 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:80" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="52" t="s">
+    <row r="5" spans="2:80" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="42" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="8" t="s">
@@ -8165,7 +8171,7 @@
       <c r="M5" s="14">
         <v>82.58</v>
       </c>
-      <c r="AA5" s="42" t="s">
+      <c r="AA5" s="45" t="s">
         <v>13</v>
       </c>
       <c r="AB5" s="12" t="s">
@@ -8189,7 +8195,7 @@
       <c r="AL5" s="20">
         <v>19.14</v>
       </c>
-      <c r="AO5" s="42" t="s">
+      <c r="AO5" s="45" t="s">
         <v>13</v>
       </c>
       <c r="AP5" s="12" t="s">
@@ -8213,7 +8219,7 @@
       <c r="AZ5" s="20">
         <v>19.829999999999998</v>
       </c>
-      <c r="BC5" s="42" t="s">
+      <c r="BC5" s="45" t="s">
         <v>13</v>
       </c>
       <c r="BD5" s="12" t="s">
@@ -8237,7 +8243,7 @@
       <c r="BN5" s="20">
         <v>20.05</v>
       </c>
-      <c r="BQ5" s="42" t="s">
+      <c r="BQ5" s="45" t="s">
         <v>13</v>
       </c>
       <c r="BR5" s="12" t="s">
@@ -8262,7 +8268,7 @@
         <v>20.92</v>
       </c>
     </row>
-    <row r="6" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B6" s="43"/>
       <c r="C6" s="9" t="s">
         <v>11</v>
@@ -8386,8 +8392,8 @@
         <v>20.92</v>
       </c>
     </row>
-    <row r="7" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="53"/>
+    <row r="7" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B7" s="44"/>
       <c r="C7" s="11" t="s">
         <v>12</v>
       </c>
@@ -8510,24 +8516,24 @@
         <v>20.49</v>
       </c>
     </row>
-    <row r="8" spans="2:80" ht="15.6" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="42" t="s">
+    <row r="8" spans="2:80" ht="15.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B8" s="45" t="s">
         <v>13</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>10</v>
       </c>
       <c r="D8" s="19">
-        <v>63.4</v>
+        <v>76.11</v>
       </c>
       <c r="E8" s="20">
-        <v>27.09</v>
+        <v>33.9</v>
       </c>
       <c r="F8" s="19">
-        <v>80.95</v>
+        <v>90.04</v>
       </c>
       <c r="G8" s="20">
-        <v>14.95</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="H8" s="19">
         <v>3.33</v>
@@ -8547,7 +8553,7 @@
       <c r="M8" s="20">
         <v>44.62</v>
       </c>
-      <c r="AA8" s="44"/>
+      <c r="AA8" s="46"/>
       <c r="AB8" s="10" t="s">
         <v>14</v>
       </c>
@@ -8569,7 +8575,7 @@
       <c r="AL8" s="22">
         <v>21.78</v>
       </c>
-      <c r="AO8" s="44"/>
+      <c r="AO8" s="46"/>
       <c r="AP8" s="10" t="s">
         <v>14</v>
       </c>
@@ -8591,7 +8597,7 @@
       <c r="AZ8" s="22">
         <v>19.12</v>
       </c>
-      <c r="BC8" s="44"/>
+      <c r="BC8" s="46"/>
       <c r="BD8" s="10" t="s">
         <v>14</v>
       </c>
@@ -8613,7 +8619,7 @@
       <c r="BN8" s="22">
         <v>19.13</v>
       </c>
-      <c r="BQ8" s="44"/>
+      <c r="BQ8" s="46"/>
       <c r="BR8" s="10" t="s">
         <v>14</v>
       </c>
@@ -8636,7 +8642,7 @@
         <v>19.53</v>
       </c>
     </row>
-    <row r="9" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B9" s="43"/>
       <c r="C9" s="9" t="s">
         <v>11</v>
@@ -8672,22 +8678,22 @@
         <v>19.09</v>
       </c>
     </row>
-    <row r="10" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B10" s="43"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D10" s="15">
-        <v>66.59</v>
+        <v>75.739999999999995</v>
       </c>
       <c r="E10" s="16">
-        <v>26.18</v>
+        <v>33.6</v>
       </c>
       <c r="F10" s="15">
         <v>84.36</v>
       </c>
       <c r="G10" s="16">
-        <v>11.95</v>
+        <v>0.68</v>
       </c>
       <c r="H10" s="15">
         <v>5.58</v>
@@ -8708,8 +8714,8 @@
         <v>44.12</v>
       </c>
     </row>
-    <row r="11" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="44"/>
+    <row r="11" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B11" s="46"/>
       <c r="C11" s="10" t="s">
         <v>14</v>
       </c>
@@ -8743,154 +8749,154 @@
       <c r="M11" s="22">
         <v>17.579999999999998</v>
       </c>
-      <c r="AA11" s="45" t="s">
+      <c r="AA11" s="47" t="s">
         <v>42</v>
       </c>
-      <c r="AB11" s="46"/>
-      <c r="AC11" s="46"/>
-      <c r="AD11" s="46"/>
-      <c r="AE11" s="46"/>
-      <c r="AF11" s="46"/>
-      <c r="AG11" s="46"/>
-      <c r="AH11" s="46"/>
-      <c r="AI11" s="46"/>
-      <c r="AJ11" s="46"/>
-      <c r="AK11" s="46"/>
-      <c r="AL11" s="47"/>
-      <c r="AO11" s="45" t="s">
+      <c r="AB11" s="48"/>
+      <c r="AC11" s="48"/>
+      <c r="AD11" s="48"/>
+      <c r="AE11" s="48"/>
+      <c r="AF11" s="48"/>
+      <c r="AG11" s="48"/>
+      <c r="AH11" s="48"/>
+      <c r="AI11" s="48"/>
+      <c r="AJ11" s="48"/>
+      <c r="AK11" s="48"/>
+      <c r="AL11" s="49"/>
+      <c r="AO11" s="47" t="s">
         <v>44</v>
       </c>
-      <c r="AP11" s="46"/>
-      <c r="AQ11" s="46"/>
-      <c r="AR11" s="46"/>
-      <c r="AS11" s="46"/>
-      <c r="AT11" s="46"/>
-      <c r="AU11" s="46"/>
-      <c r="AV11" s="46"/>
-      <c r="AW11" s="46"/>
-      <c r="AX11" s="46"/>
-      <c r="AY11" s="46"/>
-      <c r="AZ11" s="47"/>
-      <c r="BC11" s="45" t="s">
+      <c r="AP11" s="48"/>
+      <c r="AQ11" s="48"/>
+      <c r="AR11" s="48"/>
+      <c r="AS11" s="48"/>
+      <c r="AT11" s="48"/>
+      <c r="AU11" s="48"/>
+      <c r="AV11" s="48"/>
+      <c r="AW11" s="48"/>
+      <c r="AX11" s="48"/>
+      <c r="AY11" s="48"/>
+      <c r="AZ11" s="49"/>
+      <c r="BC11" s="47" t="s">
         <v>46</v>
       </c>
-      <c r="BD11" s="46"/>
-      <c r="BE11" s="46"/>
-      <c r="BF11" s="46"/>
-      <c r="BG11" s="46"/>
-      <c r="BH11" s="46"/>
-      <c r="BI11" s="46"/>
-      <c r="BJ11" s="46"/>
-      <c r="BK11" s="46"/>
-      <c r="BL11" s="46"/>
-      <c r="BM11" s="46"/>
-      <c r="BN11" s="47"/>
-      <c r="BQ11" s="45" t="s">
+      <c r="BD11" s="48"/>
+      <c r="BE11" s="48"/>
+      <c r="BF11" s="48"/>
+      <c r="BG11" s="48"/>
+      <c r="BH11" s="48"/>
+      <c r="BI11" s="48"/>
+      <c r="BJ11" s="48"/>
+      <c r="BK11" s="48"/>
+      <c r="BL11" s="48"/>
+      <c r="BM11" s="48"/>
+      <c r="BN11" s="49"/>
+      <c r="BQ11" s="47" t="s">
         <v>48</v>
       </c>
-      <c r="BR11" s="46"/>
-      <c r="BS11" s="46"/>
-      <c r="BT11" s="46"/>
-      <c r="BU11" s="46"/>
-      <c r="BV11" s="46"/>
-      <c r="BW11" s="46"/>
-      <c r="BX11" s="46"/>
-      <c r="BY11" s="46"/>
-      <c r="BZ11" s="46"/>
-      <c r="CA11" s="46"/>
-      <c r="CB11" s="47"/>
+      <c r="BR11" s="48"/>
+      <c r="BS11" s="48"/>
+      <c r="BT11" s="48"/>
+      <c r="BU11" s="48"/>
+      <c r="BV11" s="48"/>
+      <c r="BW11" s="48"/>
+      <c r="BX11" s="48"/>
+      <c r="BY11" s="48"/>
+      <c r="BZ11" s="48"/>
+      <c r="CA11" s="48"/>
+      <c r="CB11" s="49"/>
     </row>
-    <row r="12" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="AA12" s="24"/>
       <c r="AB12" s="4"/>
-      <c r="AC12" s="48" t="s">
+      <c r="AC12" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="AD12" s="49"/>
-      <c r="AE12" s="48" t="s">
+      <c r="AD12" s="51"/>
+      <c r="AE12" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="AF12" s="49"/>
-      <c r="AG12" s="48" t="s">
+      <c r="AF12" s="51"/>
+      <c r="AG12" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="AH12" s="49"/>
-      <c r="AI12" s="48" t="s">
+      <c r="AH12" s="51"/>
+      <c r="AI12" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="AJ12" s="49"/>
-      <c r="AK12" s="48" t="s">
+      <c r="AJ12" s="51"/>
+      <c r="AK12" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="AL12" s="49"/>
+      <c r="AL12" s="51"/>
       <c r="AO12" s="24"/>
       <c r="AP12" s="4"/>
-      <c r="AQ12" s="48" t="s">
+      <c r="AQ12" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="AR12" s="49"/>
-      <c r="AS12" s="48" t="s">
+      <c r="AR12" s="51"/>
+      <c r="AS12" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="AT12" s="49"/>
-      <c r="AU12" s="48" t="s">
+      <c r="AT12" s="51"/>
+      <c r="AU12" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="AV12" s="49"/>
-      <c r="AW12" s="48" t="s">
+      <c r="AV12" s="51"/>
+      <c r="AW12" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="AX12" s="49"/>
-      <c r="AY12" s="48" t="s">
+      <c r="AX12" s="51"/>
+      <c r="AY12" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="AZ12" s="49"/>
+      <c r="AZ12" s="51"/>
       <c r="BC12" s="24"/>
       <c r="BD12" s="4"/>
-      <c r="BE12" s="48" t="s">
+      <c r="BE12" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="BF12" s="49"/>
-      <c r="BG12" s="48" t="s">
+      <c r="BF12" s="51"/>
+      <c r="BG12" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="BH12" s="49"/>
-      <c r="BI12" s="48" t="s">
+      <c r="BH12" s="51"/>
+      <c r="BI12" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="BJ12" s="49"/>
-      <c r="BK12" s="48" t="s">
+      <c r="BJ12" s="51"/>
+      <c r="BK12" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="BL12" s="49"/>
-      <c r="BM12" s="48" t="s">
+      <c r="BL12" s="51"/>
+      <c r="BM12" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="BN12" s="49"/>
+      <c r="BN12" s="51"/>
       <c r="BQ12" s="24"/>
       <c r="BR12" s="4"/>
-      <c r="BS12" s="48" t="s">
+      <c r="BS12" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="BT12" s="49"/>
-      <c r="BU12" s="48" t="s">
+      <c r="BT12" s="51"/>
+      <c r="BU12" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="BV12" s="49"/>
-      <c r="BW12" s="48" t="s">
+      <c r="BV12" s="51"/>
+      <c r="BW12" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="BX12" s="49"/>
-      <c r="BY12" s="48" t="s">
+      <c r="BX12" s="51"/>
+      <c r="BY12" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="BZ12" s="49"/>
-      <c r="CA12" s="48" t="s">
+      <c r="BZ12" s="51"/>
+      <c r="CA12" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="CB12" s="49"/>
+      <c r="CB12" s="51"/>
     </row>
-    <row r="13" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="AA13" s="25" t="s">
         <v>16</v>
       </c>
@@ -9036,21 +9042,21 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="45" t="s">
+    <row r="14" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B14" s="47" t="s">
         <v>19</v>
       </c>
-      <c r="C14" s="46"/>
-      <c r="D14" s="46"/>
-      <c r="E14" s="46"/>
-      <c r="F14" s="46"/>
-      <c r="G14" s="46"/>
-      <c r="H14" s="46"/>
-      <c r="I14" s="46"/>
-      <c r="J14" s="46"/>
-      <c r="K14" s="46"/>
-      <c r="L14" s="46"/>
-      <c r="M14" s="47"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="48"/>
+      <c r="H14" s="48"/>
+      <c r="I14" s="48"/>
+      <c r="J14" s="48"/>
+      <c r="K14" s="48"/>
+      <c r="L14" s="48"/>
+      <c r="M14" s="49"/>
       <c r="AA14" s="29" t="s">
         <v>24</v>
       </c>
@@ -9112,29 +9118,29 @@
       <c r="CA14" s="30"/>
       <c r="CB14" s="30"/>
     </row>
-    <row r="15" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B15" s="24"/>
       <c r="C15" s="4"/>
-      <c r="D15" s="48" t="s">
+      <c r="D15" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="E15" s="49"/>
-      <c r="F15" s="48" t="s">
+      <c r="E15" s="51"/>
+      <c r="F15" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="G15" s="49"/>
-      <c r="H15" s="48" t="s">
+      <c r="G15" s="51"/>
+      <c r="H15" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="I15" s="49"/>
-      <c r="J15" s="48" t="s">
+      <c r="I15" s="51"/>
+      <c r="J15" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="K15" s="49"/>
-      <c r="L15" s="48" t="s">
+      <c r="K15" s="51"/>
+      <c r="L15" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="M15" s="49"/>
+      <c r="M15" s="51"/>
       <c r="AA15" s="29" t="s">
         <v>39</v>
       </c>
@@ -9192,7 +9198,7 @@
       <c r="CA15" s="30"/>
       <c r="CB15" s="30"/>
     </row>
-    <row r="16" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B16" s="25" t="s">
         <v>16</v>
       </c>
@@ -9286,24 +9292,24 @@
       <c r="CA16" s="34"/>
       <c r="CB16" s="34"/>
     </row>
-    <row r="17" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B17" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="36">
-        <v>0.77429999999999999</v>
+      <c r="C17" s="36" t="s">
+        <v>49</v>
       </c>
       <c r="D17" s="30">
-        <v>34.29</v>
+        <v>74.77</v>
       </c>
       <c r="E17" s="30">
-        <v>91.9</v>
+        <v>52.9</v>
       </c>
       <c r="F17" s="30">
-        <v>33.64</v>
+        <v>79.37</v>
       </c>
       <c r="G17" s="30">
-        <v>91.83</v>
+        <v>100</v>
       </c>
       <c r="H17" s="30">
         <v>1.08</v>
@@ -9380,22 +9386,22 @@
       <c r="CA17" s="34"/>
       <c r="CB17" s="34"/>
     </row>
-    <row r="18" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B18" s="29" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C18" s="30"/>
       <c r="D18" s="30">
-        <v>42.38</v>
+        <v>74.209999999999994</v>
       </c>
       <c r="E18" s="30">
-        <v>89.39</v>
+        <v>52.9</v>
       </c>
       <c r="F18" s="30">
-        <v>60.22</v>
+        <v>81.89</v>
       </c>
       <c r="G18" s="30">
-        <v>82.2</v>
+        <v>2.16</v>
       </c>
       <c r="H18" s="30">
         <v>1.86</v>
@@ -9472,22 +9478,22 @@
       <c r="CA18" s="30"/>
       <c r="CB18" s="30"/>
     </row>
-    <row r="19" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B19" s="29" t="s">
         <v>20</v>
       </c>
       <c r="C19" s="34"/>
       <c r="D19" s="34">
-        <v>54.02</v>
+        <v>73.64</v>
       </c>
       <c r="E19" s="34">
-        <v>30.4</v>
+        <v>53.37</v>
       </c>
       <c r="F19" s="34">
-        <v>75.39</v>
+        <v>88.05</v>
       </c>
       <c r="G19" s="34">
-        <v>26.43</v>
+        <v>0.61</v>
       </c>
       <c r="H19" s="34">
         <v>2.44</v>
@@ -9564,22 +9570,22 @@
       <c r="CA19" s="30"/>
       <c r="CB19" s="30"/>
     </row>
-    <row r="20" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B20" s="29" t="s">
         <v>29</v>
       </c>
       <c r="C20" s="34"/>
       <c r="D20" s="34">
-        <v>58.57</v>
+        <v>73.27</v>
       </c>
       <c r="E20" s="34">
-        <v>28.71</v>
+        <v>47.2</v>
       </c>
       <c r="F20" s="34">
-        <v>78.2</v>
+        <v>89.79</v>
       </c>
       <c r="G20" s="34">
-        <v>17.52</v>
+        <v>0.54</v>
       </c>
       <c r="H20" s="34">
         <v>2.82</v>
@@ -9656,22 +9662,22 @@
       <c r="CA20" s="34"/>
       <c r="CB20" s="34"/>
     </row>
-    <row r="21" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B21" s="29" t="s">
         <v>25</v>
       </c>
       <c r="C21" s="30"/>
       <c r="D21" s="30">
-        <v>61.18</v>
+        <v>72.95</v>
       </c>
       <c r="E21" s="30">
-        <v>28.38</v>
+        <v>47.26</v>
       </c>
       <c r="F21" s="30">
-        <v>78.75</v>
+        <v>89.9</v>
       </c>
       <c r="G21" s="30">
-        <v>16.989999999999998</v>
+        <v>0.54</v>
       </c>
       <c r="H21" s="30">
         <v>2.91</v>
@@ -9748,22 +9754,22 @@
       <c r="CA21" s="30"/>
       <c r="CB21" s="30"/>
     </row>
-    <row r="22" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B22" s="29" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="30"/>
       <c r="D22" s="30">
-        <v>63.4</v>
+        <v>73.849999999999994</v>
       </c>
       <c r="E22" s="30">
-        <v>27.09</v>
+        <v>33.659999999999997</v>
       </c>
       <c r="F22" s="35">
-        <v>80.95</v>
+        <v>90.08</v>
       </c>
       <c r="G22" s="30">
-        <v>14.95</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="H22" s="30">
         <v>3.33</v>
@@ -9836,22 +9842,22 @@
       <c r="CA22" s="30"/>
       <c r="CB22" s="30"/>
     </row>
-    <row r="23" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B23" s="29" t="s">
         <v>30</v>
       </c>
       <c r="C23" s="34"/>
       <c r="D23" s="34">
-        <v>64.28</v>
+        <v>74.3</v>
       </c>
       <c r="E23" s="34">
-        <v>26.47</v>
+        <v>29.93</v>
       </c>
       <c r="F23" s="34">
-        <v>82</v>
+        <v>89.98</v>
       </c>
       <c r="G23" s="34">
-        <v>14.28</v>
+        <v>0.62</v>
       </c>
       <c r="H23" s="34">
         <v>3.58</v>
@@ -9928,22 +9934,22 @@
       <c r="CA23" s="30"/>
       <c r="CB23" s="30"/>
     </row>
-    <row r="24" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B24" s="29" t="s">
         <v>26</v>
       </c>
       <c r="C24" s="30"/>
       <c r="D24" s="30">
-        <v>65.13</v>
+        <v>74.650000000000006</v>
       </c>
       <c r="E24" s="30">
-        <v>25.89</v>
+        <v>27.46</v>
       </c>
       <c r="F24" s="30">
-        <v>82.96</v>
+        <v>89.67</v>
       </c>
       <c r="G24" s="30">
-        <v>10.92</v>
+        <v>0.68</v>
       </c>
       <c r="H24" s="30">
         <v>3.84</v>
@@ -10052,22 +10058,22 @@
         <v>25.74</v>
       </c>
     </row>
-    <row r="25" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B25" s="29" t="s">
         <v>22</v>
       </c>
       <c r="C25" s="30"/>
       <c r="D25" s="30">
-        <v>67.64</v>
+        <v>75.36</v>
       </c>
       <c r="E25" s="30">
-        <v>24.34</v>
+        <v>23.22</v>
       </c>
       <c r="F25">
-        <v>85.28</v>
+        <v>84.83</v>
       </c>
       <c r="G25" s="30">
-        <v>11.74</v>
+        <v>100</v>
       </c>
       <c r="H25" s="30">
         <v>4.7699999999999996</v>
@@ -10177,22 +10183,22 @@
         <v>22.59</v>
       </c>
     </row>
-    <row r="26" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B26" s="29" t="s">
         <v>23</v>
       </c>
       <c r="C26" s="30"/>
       <c r="D26" s="30">
-        <v>75.12</v>
+        <v>79.150000000000006</v>
       </c>
       <c r="E26" s="30">
-        <v>9.82</v>
+        <v>11.57</v>
       </c>
       <c r="F26" s="30">
-        <v>88.12</v>
+        <v>72.66</v>
       </c>
       <c r="G26" s="30">
-        <v>12.57</v>
+        <v>100</v>
       </c>
       <c r="H26" s="30">
         <v>6.37</v>
@@ -10269,22 +10275,22 @@
       <c r="CA26" s="30"/>
       <c r="CB26" s="30"/>
     </row>
-    <row r="27" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B27" s="29" t="s">
         <v>31</v>
       </c>
       <c r="C27" s="30"/>
       <c r="D27" s="30">
-        <v>79.900000000000006</v>
+        <v>83.99</v>
       </c>
       <c r="E27" s="30">
-        <v>6.72</v>
+        <v>4.24</v>
       </c>
       <c r="F27" s="30">
-        <v>90.94</v>
+        <v>63.45</v>
       </c>
       <c r="G27" s="30">
-        <v>15.04</v>
+        <v>100</v>
       </c>
       <c r="H27" s="30">
         <v>7.68</v>
@@ -10393,22 +10399,22 @@
         <v>64.8</v>
       </c>
     </row>
-    <row r="28" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B28" s="29" t="s">
         <v>40</v>
       </c>
       <c r="C28" s="30"/>
       <c r="D28" s="30">
-        <v>82.66</v>
+        <v>84.35</v>
       </c>
       <c r="E28" s="30">
-        <v>4.93</v>
+        <v>3.64</v>
       </c>
       <c r="F28" s="30">
-        <v>91</v>
+        <v>56.31</v>
       </c>
       <c r="G28" s="30">
-        <v>16.91</v>
+        <v>100</v>
       </c>
       <c r="H28" s="30">
         <v>7.94</v>
@@ -10485,22 +10491,22 @@
       <c r="CA28" s="30"/>
       <c r="CB28" s="30"/>
     </row>
-    <row r="29" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B29" s="29" t="s">
         <v>27</v>
       </c>
       <c r="C29" s="30"/>
       <c r="D29" s="30">
-        <v>83.9</v>
+        <v>84.2</v>
       </c>
       <c r="E29" s="30">
-        <v>3.91</v>
+        <v>3.52</v>
       </c>
       <c r="F29" s="30">
-        <v>91.17</v>
+        <v>51.7</v>
       </c>
       <c r="G29" s="30">
-        <v>17.68</v>
+        <v>100</v>
       </c>
       <c r="H29" s="30">
         <v>7.97</v>
@@ -10609,22 +10615,22 @@
         <v>93.76</v>
       </c>
     </row>
-    <row r="30" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B30" s="29" t="s">
         <v>32</v>
       </c>
       <c r="C30" s="30"/>
       <c r="D30" s="30">
-        <v>84.85</v>
+        <v>83.5</v>
       </c>
       <c r="E30" s="30">
-        <v>3.18</v>
+        <v>3.6</v>
       </c>
       <c r="F30" s="30">
-        <v>91.29</v>
+        <v>45.62</v>
       </c>
       <c r="G30" s="30">
-        <v>19.440000000000001</v>
+        <v>100</v>
       </c>
       <c r="H30" s="30">
         <v>7.91</v>
@@ -10733,22 +10739,22 @@
         <v>93.93</v>
       </c>
     </row>
-    <row r="31" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B31" s="29" t="s">
         <v>28</v>
       </c>
       <c r="C31" s="30"/>
       <c r="D31" s="30">
-        <v>85.12</v>
+        <v>82.83</v>
       </c>
       <c r="E31" s="30">
-        <v>2.97</v>
+        <v>3.73</v>
       </c>
       <c r="F31" s="30">
-        <v>91.31</v>
+        <v>42.33</v>
       </c>
       <c r="G31" s="30">
-        <v>20.47</v>
+        <v>100</v>
       </c>
       <c r="H31" s="30">
         <v>7.86</v>
@@ -10857,22 +10863,22 @@
         <v>94.03</v>
       </c>
     </row>
-    <row r="32" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B32" s="29" t="s">
         <v>33</v>
       </c>
       <c r="C32" s="30"/>
       <c r="D32" s="30">
-        <v>85.25</v>
+        <v>82.29</v>
       </c>
       <c r="E32" s="30">
-        <v>2.86</v>
+        <v>3.84</v>
       </c>
       <c r="F32" s="30">
-        <v>91.31</v>
+        <v>39.26</v>
       </c>
       <c r="G32" s="30">
-        <v>21.04</v>
+        <v>100</v>
       </c>
       <c r="H32" s="30">
         <v>7.82</v>
@@ -10981,22 +10987,22 @@
         <v>94.09</v>
       </c>
     </row>
-    <row r="33" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B33" s="29" t="s">
         <v>34</v>
       </c>
       <c r="C33" s="30"/>
       <c r="D33" s="30">
-        <v>85.33</v>
+        <v>81.849999999999994</v>
       </c>
       <c r="E33" s="30">
-        <v>2.8</v>
+        <v>3.93</v>
       </c>
       <c r="F33" s="30">
-        <v>91.31</v>
+        <v>37.42</v>
       </c>
       <c r="G33" s="30">
-        <v>21.37</v>
+        <v>100</v>
       </c>
       <c r="H33" s="30">
         <v>7.79</v>
@@ -11105,22 +11111,22 @@
         <v>94.13</v>
       </c>
     </row>
-    <row r="34" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B34" s="29" t="s">
         <v>35</v>
       </c>
       <c r="C34" s="30"/>
       <c r="D34" s="30">
-        <v>85.38</v>
+        <v>81.5</v>
       </c>
       <c r="E34" s="30">
-        <v>2.76</v>
+        <v>4</v>
       </c>
       <c r="F34" s="30">
-        <v>91.3</v>
+        <v>36.72</v>
       </c>
       <c r="G34" s="30">
-        <v>21.52</v>
+        <v>100</v>
       </c>
       <c r="H34" s="30">
         <v>7.77</v>
@@ -11229,22 +11235,22 @@
         <v>94.16</v>
       </c>
     </row>
-    <row r="35" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B35" s="29" t="s">
         <v>36</v>
       </c>
       <c r="C35" s="30"/>
       <c r="D35" s="30">
-        <v>85.42</v>
+        <v>81.2</v>
       </c>
       <c r="E35" s="30">
-        <v>2.73</v>
+        <v>4.07</v>
       </c>
       <c r="F35" s="30">
-        <v>91.3</v>
+        <v>36.28</v>
       </c>
       <c r="G35" s="30">
-        <v>21.62</v>
+        <v>100</v>
       </c>
       <c r="H35" s="30">
         <v>7.76</v>
@@ -11317,22 +11323,22 @@
       <c r="CA35" s="38"/>
       <c r="CB35" s="39"/>
     </row>
-    <row r="36" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B36" s="29" t="s">
         <v>37</v>
       </c>
       <c r="C36" s="30"/>
       <c r="D36" s="30">
-        <v>85.45</v>
+        <v>80.95</v>
       </c>
       <c r="E36" s="30">
-        <v>2.7</v>
+        <v>4.12</v>
       </c>
       <c r="F36" s="30">
-        <v>91.3</v>
+        <v>35.979999999999997</v>
       </c>
       <c r="G36" s="30">
-        <v>21.75</v>
+        <v>100</v>
       </c>
       <c r="H36" s="30">
         <v>7.75</v>
@@ -11353,22 +11359,22 @@
         <v>41.32</v>
       </c>
     </row>
-    <row r="37" spans="2:80" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:80" x14ac:dyDescent="0.35">
       <c r="B37" s="29" t="s">
         <v>38</v>
       </c>
       <c r="C37" s="30"/>
       <c r="D37" s="30">
-        <v>85.47</v>
+        <v>80.7</v>
       </c>
       <c r="E37" s="30">
-        <v>2.68</v>
+        <v>4.1900000000000004</v>
       </c>
       <c r="F37" s="37">
-        <v>91.29</v>
+        <v>35.75</v>
       </c>
       <c r="G37" s="30">
-        <v>21.84</v>
+        <v>100</v>
       </c>
       <c r="H37" s="30">
         <v>7.74</v>
@@ -11389,7 +11395,7 @@
         <v>41.43</v>
       </c>
     </row>
-    <row r="38" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="2:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="C38" s="23" t="s">
         <v>17</v>
       </c>
@@ -11406,11 +11412,84 @@
     </row>
   </sheetData>
   <mergeCells count="91">
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="J38:K38"/>
-    <mergeCell ref="L38:M38"/>
+    <mergeCell ref="BS35:BT35"/>
+    <mergeCell ref="BU35:BV35"/>
+    <mergeCell ref="BW35:BX35"/>
+    <mergeCell ref="BY35:BZ35"/>
+    <mergeCell ref="CA35:CB35"/>
+    <mergeCell ref="BQ5:BQ8"/>
+    <mergeCell ref="BQ11:CB11"/>
+    <mergeCell ref="BS12:BT12"/>
+    <mergeCell ref="BU12:BV12"/>
+    <mergeCell ref="BW12:BX12"/>
+    <mergeCell ref="BY12:BZ12"/>
+    <mergeCell ref="CA12:CB12"/>
+    <mergeCell ref="BQ2:CB2"/>
+    <mergeCell ref="BS3:BT3"/>
+    <mergeCell ref="BU3:BV3"/>
+    <mergeCell ref="BW3:BX3"/>
+    <mergeCell ref="BY3:BZ3"/>
+    <mergeCell ref="CA3:CB3"/>
+    <mergeCell ref="BE35:BF35"/>
+    <mergeCell ref="BG35:BH35"/>
+    <mergeCell ref="BI35:BJ35"/>
+    <mergeCell ref="BK35:BL35"/>
+    <mergeCell ref="BM35:BN35"/>
+    <mergeCell ref="BC5:BC8"/>
+    <mergeCell ref="BC11:BN11"/>
+    <mergeCell ref="BE12:BF12"/>
+    <mergeCell ref="BG12:BH12"/>
+    <mergeCell ref="BI12:BJ12"/>
+    <mergeCell ref="BK12:BL12"/>
+    <mergeCell ref="BM12:BN12"/>
+    <mergeCell ref="BC2:BN2"/>
+    <mergeCell ref="BE3:BF3"/>
+    <mergeCell ref="BG3:BH3"/>
+    <mergeCell ref="BI3:BJ3"/>
+    <mergeCell ref="BK3:BL3"/>
+    <mergeCell ref="BM3:BN3"/>
+    <mergeCell ref="AQ35:AR35"/>
+    <mergeCell ref="AS35:AT35"/>
+    <mergeCell ref="AU35:AV35"/>
+    <mergeCell ref="AW35:AX35"/>
+    <mergeCell ref="AY35:AZ35"/>
+    <mergeCell ref="AO5:AO8"/>
+    <mergeCell ref="AO11:AZ11"/>
+    <mergeCell ref="AQ12:AR12"/>
+    <mergeCell ref="AS12:AT12"/>
+    <mergeCell ref="AU12:AV12"/>
+    <mergeCell ref="AW12:AX12"/>
+    <mergeCell ref="AY12:AZ12"/>
+    <mergeCell ref="AO2:AZ2"/>
+    <mergeCell ref="AQ3:AR3"/>
+    <mergeCell ref="AS3:AT3"/>
+    <mergeCell ref="AU3:AV3"/>
+    <mergeCell ref="AW3:AX3"/>
+    <mergeCell ref="AY3:AZ3"/>
+    <mergeCell ref="AC35:AD35"/>
+    <mergeCell ref="AE35:AF35"/>
+    <mergeCell ref="AG35:AH35"/>
+    <mergeCell ref="AI35:AJ35"/>
+    <mergeCell ref="AK35:AL35"/>
+    <mergeCell ref="AA5:AA8"/>
+    <mergeCell ref="AA11:AL11"/>
+    <mergeCell ref="AC12:AD12"/>
+    <mergeCell ref="AE12:AF12"/>
+    <mergeCell ref="AG12:AH12"/>
+    <mergeCell ref="AI12:AJ12"/>
+    <mergeCell ref="AK12:AL12"/>
+    <mergeCell ref="AA2:AL2"/>
+    <mergeCell ref="AC3:AD3"/>
+    <mergeCell ref="AE3:AF3"/>
+    <mergeCell ref="AG3:AH3"/>
+    <mergeCell ref="AI3:AJ3"/>
+    <mergeCell ref="AK3:AL3"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="D3:E3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="L3:M3"/>
     <mergeCell ref="B5:B7"/>
     <mergeCell ref="B8:B11"/>
     <mergeCell ref="B14:M14"/>
@@ -11419,84 +11498,11 @@
     <mergeCell ref="H15:I15"/>
     <mergeCell ref="J15:K15"/>
     <mergeCell ref="L15:M15"/>
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="L3:M3"/>
-    <mergeCell ref="AA2:AL2"/>
-    <mergeCell ref="AC3:AD3"/>
-    <mergeCell ref="AE3:AF3"/>
-    <mergeCell ref="AG3:AH3"/>
-    <mergeCell ref="AI3:AJ3"/>
-    <mergeCell ref="AK3:AL3"/>
-    <mergeCell ref="AA5:AA8"/>
-    <mergeCell ref="AA11:AL11"/>
-    <mergeCell ref="AC12:AD12"/>
-    <mergeCell ref="AE12:AF12"/>
-    <mergeCell ref="AG12:AH12"/>
-    <mergeCell ref="AI12:AJ12"/>
-    <mergeCell ref="AK12:AL12"/>
-    <mergeCell ref="AC35:AD35"/>
-    <mergeCell ref="AE35:AF35"/>
-    <mergeCell ref="AG35:AH35"/>
-    <mergeCell ref="AI35:AJ35"/>
-    <mergeCell ref="AK35:AL35"/>
-    <mergeCell ref="AO2:AZ2"/>
-    <mergeCell ref="AQ3:AR3"/>
-    <mergeCell ref="AS3:AT3"/>
-    <mergeCell ref="AU3:AV3"/>
-    <mergeCell ref="AW3:AX3"/>
-    <mergeCell ref="AY3:AZ3"/>
-    <mergeCell ref="AO5:AO8"/>
-    <mergeCell ref="AO11:AZ11"/>
-    <mergeCell ref="AQ12:AR12"/>
-    <mergeCell ref="AS12:AT12"/>
-    <mergeCell ref="AU12:AV12"/>
-    <mergeCell ref="AW12:AX12"/>
-    <mergeCell ref="AY12:AZ12"/>
-    <mergeCell ref="AQ35:AR35"/>
-    <mergeCell ref="AS35:AT35"/>
-    <mergeCell ref="AU35:AV35"/>
-    <mergeCell ref="AW35:AX35"/>
-    <mergeCell ref="AY35:AZ35"/>
-    <mergeCell ref="BC2:BN2"/>
-    <mergeCell ref="BE3:BF3"/>
-    <mergeCell ref="BG3:BH3"/>
-    <mergeCell ref="BI3:BJ3"/>
-    <mergeCell ref="BK3:BL3"/>
-    <mergeCell ref="BM3:BN3"/>
-    <mergeCell ref="BC5:BC8"/>
-    <mergeCell ref="BC11:BN11"/>
-    <mergeCell ref="BE12:BF12"/>
-    <mergeCell ref="BG12:BH12"/>
-    <mergeCell ref="BI12:BJ12"/>
-    <mergeCell ref="BK12:BL12"/>
-    <mergeCell ref="BM12:BN12"/>
-    <mergeCell ref="BE35:BF35"/>
-    <mergeCell ref="BG35:BH35"/>
-    <mergeCell ref="BI35:BJ35"/>
-    <mergeCell ref="BK35:BL35"/>
-    <mergeCell ref="BM35:BN35"/>
-    <mergeCell ref="BQ2:CB2"/>
-    <mergeCell ref="BS3:BT3"/>
-    <mergeCell ref="BU3:BV3"/>
-    <mergeCell ref="BW3:BX3"/>
-    <mergeCell ref="BY3:BZ3"/>
-    <mergeCell ref="CA3:CB3"/>
-    <mergeCell ref="BQ5:BQ8"/>
-    <mergeCell ref="BQ11:CB11"/>
-    <mergeCell ref="BS12:BT12"/>
-    <mergeCell ref="BU12:BV12"/>
-    <mergeCell ref="BW12:BX12"/>
-    <mergeCell ref="BY12:BZ12"/>
-    <mergeCell ref="CA12:CB12"/>
-    <mergeCell ref="BS35:BT35"/>
-    <mergeCell ref="BU35:BV35"/>
-    <mergeCell ref="BW35:BX35"/>
-    <mergeCell ref="BY35:BZ35"/>
-    <mergeCell ref="CA35:CB35"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="L38:M38"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
terzo vett temp lf
</commit_message>
<xml_diff>
--- a/Results_metrics.xlsx
+++ b/Results_metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ludovicascaffidi/Desktop/Università/Magistrale/Secondo Anno/Secondo Semestre/Machine Learning for Mathematical Engineering/Progetto/MaskArchitectureAnomaly_CourseProject/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a8875455940b8c0f/Desktop/UNI/MACHINE LEARNING/Progetto/MaskArchitectureAnomaly_CourseProject/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E602311C-DCBC-F649-AD7D-8F8F41C583C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{E602311C-DCBC-F649-AD7D-8F8F41C583C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DEB2989-C1CF-4D72-BB4E-D1E39A7C3C83}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4220" yWindow="620" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -199,7 +199,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,6 +235,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Calibri "/>
     </font>
   </fonts>
   <fills count="8">
@@ -698,7 +703,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
@@ -786,6 +791,7 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -1530,6 +1536,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1537,7 +1544,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2299,6 +2305,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2306,7 +2313,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -2557,6 +2563,27 @@
                 <c:pt idx="6">
                   <c:v>25.8</c:v>
                 </c:pt>
+                <c:pt idx="7">
+                  <c:v>26.09</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>26.67</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>27.15</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>27.59</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>27.96</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>28.28</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>28.74</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -2702,6 +2729,27 @@
                 </c:pt>
                 <c:pt idx="6">
                   <c:v>14.93</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>15.37</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>15.61</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>13.71</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>16.43</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>16.16</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>16.940000000000001</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>29.06</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2984,6 +3032,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2991,7 +3040,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3753,6 +3801,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -3760,7 +3809,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4486,6 +4534,7 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4493,7 +4542,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7436,6 +7484,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -7700,19 +7752,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B1:CP107"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5"/>
   <cols>
-    <col min="2" max="2" width="14.5" customWidth="1"/>
-    <col min="3" max="3" width="13.1640625" customWidth="1"/>
-    <col min="28" max="28" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.453125" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" customWidth="1"/>
+    <col min="28" max="28" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="12.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:94" ht="15" thickBot="1"/>
+    <row r="2" spans="2:94" ht="15" thickBot="1">
       <c r="B2" s="45" t="s">
         <v>18</v>
       </c>
@@ -7798,7 +7850,7 @@
       <c r="CO2" s="51"/>
       <c r="CP2" s="52"/>
     </row>
-    <row r="3" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:94" ht="15" thickBot="1">
       <c r="B3" s="1"/>
       <c r="C3" s="5"/>
       <c r="D3" s="43" t="s">
@@ -7942,7 +7994,7 @@
       </c>
       <c r="CP3" s="44"/>
     </row>
-    <row r="4" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:94" ht="15" thickBot="1">
       <c r="B4" s="6" t="s">
         <v>0</v>
       </c>
@@ -8160,7 +8212,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="2:94" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:94" ht="15" thickTop="1">
       <c r="B5" s="53" t="s">
         <v>9</v>
       </c>
@@ -8278,7 +8330,7 @@
       <c r="CO5" s="19"/>
       <c r="CP5" s="20"/>
     </row>
-    <row r="6" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:94">
       <c r="B6" s="49"/>
       <c r="C6" s="9" t="s">
         <v>11</v>
@@ -8384,7 +8436,7 @@
       <c r="CO6" s="15"/>
       <c r="CP6" s="16"/>
     </row>
-    <row r="7" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:94" ht="15" thickBot="1">
       <c r="B7" s="54"/>
       <c r="C7" s="11" t="s">
         <v>12</v>
@@ -8490,7 +8542,7 @@
       <c r="CO7" s="15"/>
       <c r="CP7" s="16"/>
     </row>
-    <row r="8" spans="2:94" ht="17" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:94" ht="15.5" thickTop="1" thickBot="1">
       <c r="B8" s="48" t="s">
         <v>13</v>
       </c>
@@ -8598,7 +8650,7 @@
       <c r="CO8" s="21"/>
       <c r="CP8" s="22"/>
     </row>
-    <row r="9" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:94">
       <c r="B9" s="49"/>
       <c r="C9" s="9" t="s">
         <v>11</v>
@@ -8634,7 +8686,7 @@
         <v>19.09</v>
       </c>
     </row>
-    <row r="10" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:94" ht="15" thickBot="1">
       <c r="B10" s="49"/>
       <c r="C10" s="9" t="s">
         <v>12</v>
@@ -8670,7 +8722,7 @@
         <v>18.829999999999998</v>
       </c>
     </row>
-    <row r="11" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:94" ht="15" thickBot="1">
       <c r="B11" s="50"/>
       <c r="C11" s="10" t="s">
         <v>14</v>
@@ -8776,7 +8828,7 @@
       <c r="CO11" s="46"/>
       <c r="CP11" s="47"/>
     </row>
-    <row r="12" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:94" ht="15" thickBot="1">
       <c r="AA12" s="24"/>
       <c r="AB12" s="5" t="s">
         <v>53</v>
@@ -8898,7 +8950,7 @@
       </c>
       <c r="CP12" s="44"/>
     </row>
-    <row r="13" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:94" ht="15" thickBot="1">
       <c r="AA13" s="25" t="s">
         <v>16</v>
       </c>
@@ -9080,7 +9132,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:94" ht="15" thickBot="1">
       <c r="B14" s="45" t="s">
         <v>19</v>
       </c>
@@ -9166,7 +9218,7 @@
       <c r="CO14" s="30"/>
       <c r="CP14" s="30"/>
     </row>
-    <row r="15" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:94" ht="15" thickBot="1">
       <c r="B15" s="24"/>
       <c r="C15" s="4"/>
       <c r="D15" s="43" t="s">
@@ -9260,7 +9312,7 @@
       <c r="CO15" s="30"/>
       <c r="CP15" s="30"/>
     </row>
-    <row r="16" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:94">
       <c r="B16" s="25" t="s">
         <v>16</v>
       </c>
@@ -9368,7 +9420,7 @@
       <c r="CO16" s="34"/>
       <c r="CP16" s="34"/>
     </row>
-    <row r="17" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:94">
       <c r="B17" s="29" t="s">
         <v>24</v>
       </c>
@@ -9476,7 +9528,7 @@
       <c r="CO17" s="34"/>
       <c r="CP17" s="34"/>
     </row>
-    <row r="18" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:94">
       <c r="B18" s="29" t="s">
         <v>45</v>
       </c>
@@ -9582,7 +9634,7 @@
       <c r="CO18" s="30"/>
       <c r="CP18" s="30"/>
     </row>
-    <row r="19" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:94">
       <c r="B19" s="29" t="s">
         <v>20</v>
       </c>
@@ -9688,7 +9740,7 @@
       <c r="CO19" s="30"/>
       <c r="CP19" s="30"/>
     </row>
-    <row r="20" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:94">
       <c r="B20" s="29" t="s">
         <v>29</v>
       </c>
@@ -9794,7 +9846,7 @@
       <c r="CO20" s="34"/>
       <c r="CP20" s="34"/>
     </row>
-    <row r="21" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:94">
       <c r="B21" s="29" t="s">
         <v>25</v>
       </c>
@@ -9900,7 +9952,7 @@
       <c r="CO21" s="30"/>
       <c r="CP21" s="30"/>
     </row>
-    <row r="22" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:94">
       <c r="B22" s="29" t="s">
         <v>21</v>
       </c>
@@ -10001,7 +10053,7 @@
       <c r="CO22" s="30"/>
       <c r="CP22" s="30"/>
     </row>
-    <row r="23" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:94">
       <c r="B23" s="29" t="s">
         <v>30</v>
       </c>
@@ -10107,7 +10159,7 @@
       <c r="CO23" s="30"/>
       <c r="CP23" s="30"/>
     </row>
-    <row r="24" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:94">
       <c r="B24" s="29" t="s">
         <v>26</v>
       </c>
@@ -10124,8 +10176,12 @@
       <c r="G24" s="30">
         <v>0.68</v>
       </c>
-      <c r="H24" s="30"/>
-      <c r="I24" s="30"/>
+      <c r="H24" s="55">
+        <v>26.09</v>
+      </c>
+      <c r="I24" s="30">
+        <v>15.37</v>
+      </c>
       <c r="J24" s="30">
         <v>54.66</v>
       </c>
@@ -10209,7 +10265,7 @@
       <c r="CO24" s="30"/>
       <c r="CP24" s="30"/>
     </row>
-    <row r="25" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:94">
       <c r="B25" s="29" t="s">
         <v>22</v>
       </c>
@@ -10226,8 +10282,12 @@
       <c r="G25" s="30">
         <v>100</v>
       </c>
-      <c r="H25" s="30"/>
-      <c r="I25" s="30"/>
+      <c r="H25" s="30">
+        <v>26.67</v>
+      </c>
+      <c r="I25" s="30">
+        <v>15.61</v>
+      </c>
       <c r="J25" s="30">
         <v>54.68</v>
       </c>
@@ -10312,7 +10372,7 @@
       <c r="CO25" s="30"/>
       <c r="CP25" s="30"/>
     </row>
-    <row r="26" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:94">
       <c r="B26" s="29" t="s">
         <v>23</v>
       </c>
@@ -10329,8 +10389,12 @@
       <c r="G26" s="30">
         <v>100</v>
       </c>
-      <c r="H26" s="30"/>
-      <c r="I26" s="30"/>
+      <c r="H26" s="30">
+        <v>27.15</v>
+      </c>
+      <c r="I26" s="30">
+        <v>13.71</v>
+      </c>
       <c r="J26" s="30">
         <v>54.32</v>
       </c>
@@ -10414,7 +10478,7 @@
       <c r="CO26" s="30"/>
       <c r="CP26" s="30"/>
     </row>
-    <row r="27" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:94">
       <c r="B27" s="29" t="s">
         <v>31</v>
       </c>
@@ -10431,8 +10495,12 @@
       <c r="G27" s="30">
         <v>100</v>
       </c>
-      <c r="H27" s="30"/>
-      <c r="I27" s="30"/>
+      <c r="H27" s="30">
+        <v>27.59</v>
+      </c>
+      <c r="I27" s="30">
+        <v>16.43</v>
+      </c>
       <c r="J27" s="30">
         <v>53.61</v>
       </c>
@@ -10516,7 +10584,7 @@
       <c r="CO27" s="30"/>
       <c r="CP27" s="30"/>
     </row>
-    <row r="28" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:94">
       <c r="B28" s="29" t="s">
         <v>40</v>
       </c>
@@ -10533,8 +10601,12 @@
       <c r="G28" s="30">
         <v>100</v>
       </c>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
+      <c r="H28" s="30">
+        <v>27.96</v>
+      </c>
+      <c r="I28" s="30">
+        <v>16.16</v>
+      </c>
       <c r="J28" s="30">
         <v>53.44</v>
       </c>
@@ -10618,7 +10690,7 @@
       <c r="CO28" s="30"/>
       <c r="CP28" s="30"/>
     </row>
-    <row r="29" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:94">
       <c r="B29" s="29" t="s">
         <v>27</v>
       </c>
@@ -10635,8 +10707,12 @@
       <c r="G29" s="30">
         <v>100</v>
       </c>
-      <c r="H29" s="30"/>
-      <c r="I29" s="30"/>
+      <c r="H29" s="30">
+        <v>28.28</v>
+      </c>
+      <c r="I29" s="30">
+        <v>16.940000000000001</v>
+      </c>
       <c r="J29" s="30">
         <v>53.61</v>
       </c>
@@ -10720,7 +10796,7 @@
       <c r="CO29" s="30"/>
       <c r="CP29" s="30"/>
     </row>
-    <row r="30" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:94">
       <c r="B30" s="29" t="s">
         <v>32</v>
       </c>
@@ -10737,8 +10813,12 @@
       <c r="G30" s="30">
         <v>100</v>
       </c>
-      <c r="H30" s="30"/>
-      <c r="I30" s="30"/>
+      <c r="H30" s="30">
+        <v>28.74</v>
+      </c>
+      <c r="I30" s="30">
+        <v>29.06</v>
+      </c>
       <c r="J30" s="30">
         <v>54.17</v>
       </c>
@@ -10822,7 +10902,7 @@
       <c r="CO30" s="30"/>
       <c r="CP30" s="30"/>
     </row>
-    <row r="31" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:94">
       <c r="B31" s="29" t="s">
         <v>28</v>
       </c>
@@ -10924,7 +11004,7 @@
       <c r="CO31" s="30"/>
       <c r="CP31" s="30"/>
     </row>
-    <row r="32" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:94">
       <c r="B32" s="29" t="s">
         <v>33</v>
       </c>
@@ -11026,7 +11106,7 @@
       <c r="CO32" s="30"/>
       <c r="CP32" s="30"/>
     </row>
-    <row r="33" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:94">
       <c r="B33" s="29" t="s">
         <v>34</v>
       </c>
@@ -11128,7 +11208,7 @@
       <c r="CO33" s="30"/>
       <c r="CP33" s="30"/>
     </row>
-    <row r="34" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:94">
       <c r="B34" s="29" t="s">
         <v>35</v>
       </c>
@@ -11230,7 +11310,7 @@
       <c r="CO34" s="30"/>
       <c r="CP34" s="30"/>
     </row>
-    <row r="35" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:94" ht="15" thickBot="1">
       <c r="B35" s="29" t="s">
         <v>36</v>
       </c>
@@ -11327,7 +11407,7 @@
       <c r="CO35" s="39"/>
       <c r="CP35" s="40"/>
     </row>
-    <row r="36" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:94">
       <c r="B36" s="29" t="s">
         <v>37</v>
       </c>
@@ -11359,7 +11439,7 @@
         <v>13.42</v>
       </c>
     </row>
-    <row r="37" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:94" ht="15" thickBot="1">
       <c r="B37" s="29" t="s">
         <v>38</v>
       </c>
@@ -11391,7 +11471,7 @@
         <v>13.38</v>
       </c>
     </row>
-    <row r="38" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:94" ht="15" thickBot="1">
       <c r="C38" s="23" t="s">
         <v>17</v>
       </c>
@@ -11478,7 +11558,7 @@
       <c r="CO38" s="51"/>
       <c r="CP38" s="52"/>
     </row>
-    <row r="39" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:94" ht="15" thickBot="1">
       <c r="AA39" s="1"/>
       <c r="AB39" s="5" t="s">
         <v>54</v>
@@ -11600,7 +11680,7 @@
       </c>
       <c r="CP39" s="44"/>
     </row>
-    <row r="40" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:94" ht="15" thickBot="1">
       <c r="AA40" s="6" t="s">
         <v>0</v>
       </c>
@@ -11782,7 +11862,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="41" spans="2:94" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:94" ht="15" thickTop="1">
       <c r="AA41" s="48" t="s">
         <v>13</v>
       </c>
@@ -11864,7 +11944,7 @@
       <c r="CO41" s="19"/>
       <c r="CP41" s="20"/>
     </row>
-    <row r="42" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:94">
       <c r="AA42" s="49"/>
       <c r="AB42" s="9" t="s">
         <v>11</v>
@@ -11936,7 +12016,7 @@
       <c r="CO42" s="15"/>
       <c r="CP42" s="16"/>
     </row>
-    <row r="43" spans="2:94" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:94">
       <c r="AA43" s="49"/>
       <c r="AB43" s="9" t="s">
         <v>12</v>
@@ -12008,7 +12088,7 @@
       <c r="CO43" s="15"/>
       <c r="CP43" s="16"/>
     </row>
-    <row r="44" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:94" ht="15" thickBot="1">
       <c r="AA44" s="50"/>
       <c r="AB44" s="10" t="s">
         <v>14</v>
@@ -12080,8 +12160,8 @@
       <c r="CO44" s="21"/>
       <c r="CP44" s="22"/>
     </row>
-    <row r="46" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:94" ht="15" thickBot="1"/>
+    <row r="47" spans="2:94" ht="15" thickBot="1">
       <c r="AA47" s="45" t="s">
         <v>47</v>
       </c>
@@ -12153,7 +12233,7 @@
       <c r="CO47" s="46"/>
       <c r="CP47" s="47"/>
     </row>
-    <row r="48" spans="2:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:94" ht="15" thickBot="1">
       <c r="AA48" s="24"/>
       <c r="AB48" s="5" t="s">
         <v>54</v>
@@ -12275,7 +12355,7 @@
       </c>
       <c r="CP48" s="44"/>
     </row>
-    <row r="49" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="49" spans="27:94">
       <c r="AA49" s="25" t="s">
         <v>16</v>
       </c>
@@ -12457,7 +12537,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="50" spans="27:94">
       <c r="AA50" s="29" t="s">
         <v>24</v>
       </c>
@@ -12529,7 +12609,7 @@
       <c r="CO50" s="30"/>
       <c r="CP50" s="30"/>
     </row>
-    <row r="51" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="51" spans="27:94">
       <c r="AA51" s="29" t="s">
         <v>39</v>
       </c>
@@ -12601,7 +12681,7 @@
       <c r="CO51" s="30"/>
       <c r="CP51" s="30"/>
     </row>
-    <row r="52" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="52" spans="27:94">
       <c r="AA52" s="29" t="s">
         <v>20</v>
       </c>
@@ -12673,7 +12753,7 @@
       <c r="CO52" s="34"/>
       <c r="CP52" s="34"/>
     </row>
-    <row r="53" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="53" spans="27:94">
       <c r="AA53" s="29" t="s">
         <v>29</v>
       </c>
@@ -12745,7 +12825,7 @@
       <c r="CO53" s="34"/>
       <c r="CP53" s="34"/>
     </row>
-    <row r="54" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="54" spans="27:94">
       <c r="AA54" s="29" t="s">
         <v>25</v>
       </c>
@@ -12817,7 +12897,7 @@
       <c r="CO54" s="30"/>
       <c r="CP54" s="30"/>
     </row>
-    <row r="55" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="55" spans="27:94">
       <c r="AA55" s="29" t="s">
         <v>21</v>
       </c>
@@ -12889,7 +12969,7 @@
       <c r="CO55" s="30"/>
       <c r="CP55" s="30"/>
     </row>
-    <row r="56" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="56" spans="27:94">
       <c r="AA56" s="29" t="s">
         <v>30</v>
       </c>
@@ -12961,7 +13041,7 @@
       <c r="CO56" s="34"/>
       <c r="CP56" s="34"/>
     </row>
-    <row r="57" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="57" spans="27:94">
       <c r="AA57" s="29" t="s">
         <v>26</v>
       </c>
@@ -13033,7 +13113,7 @@
       <c r="CO57" s="30"/>
       <c r="CP57" s="30"/>
     </row>
-    <row r="58" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="58" spans="27:94">
       <c r="AA58" s="29" t="s">
         <v>22</v>
       </c>
@@ -13100,7 +13180,7 @@
       <c r="CO58" s="30"/>
       <c r="CP58" s="30"/>
     </row>
-    <row r="59" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="59" spans="27:94">
       <c r="AA59" s="29" t="s">
         <v>23</v>
       </c>
@@ -13172,7 +13252,7 @@
       <c r="CO59" s="30"/>
       <c r="CP59" s="30"/>
     </row>
-    <row r="60" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="60" spans="27:94">
       <c r="AA60" s="29" t="s">
         <v>31</v>
       </c>
@@ -13244,7 +13324,7 @@
       <c r="CO60" s="30"/>
       <c r="CP60" s="30"/>
     </row>
-    <row r="61" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="61" spans="27:94">
       <c r="AA61" s="29" t="s">
         <v>40</v>
       </c>
@@ -13316,7 +13396,7 @@
       <c r="CO61" s="30"/>
       <c r="CP61" s="30"/>
     </row>
-    <row r="62" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="62" spans="27:94">
       <c r="AA62" s="29" t="s">
         <v>27</v>
       </c>
@@ -13388,7 +13468,7 @@
       <c r="CO62" s="30"/>
       <c r="CP62" s="30"/>
     </row>
-    <row r="63" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="63" spans="27:94">
       <c r="AA63" s="29" t="s">
         <v>32</v>
       </c>
@@ -13460,7 +13540,7 @@
       <c r="CO63" s="30"/>
       <c r="CP63" s="30"/>
     </row>
-    <row r="64" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="64" spans="27:94">
       <c r="AA64" s="29" t="s">
         <v>28</v>
       </c>
@@ -13532,7 +13612,7 @@
       <c r="CO64" s="30"/>
       <c r="CP64" s="30"/>
     </row>
-    <row r="65" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="65" spans="27:94">
       <c r="AA65" s="29" t="s">
         <v>33</v>
       </c>
@@ -13604,7 +13684,7 @@
       <c r="CO65" s="30"/>
       <c r="CP65" s="30"/>
     </row>
-    <row r="66" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="66" spans="27:94">
       <c r="AA66" s="29" t="s">
         <v>34</v>
       </c>
@@ -13676,7 +13756,7 @@
       <c r="CO66" s="30"/>
       <c r="CP66" s="30"/>
     </row>
-    <row r="67" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="67" spans="27:94">
       <c r="AA67" s="29" t="s">
         <v>35</v>
       </c>
@@ -13748,7 +13828,7 @@
       <c r="CO67" s="30"/>
       <c r="CP67" s="30"/>
     </row>
-    <row r="68" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="68" spans="27:94">
       <c r="AA68" s="29" t="s">
         <v>36</v>
       </c>
@@ -13820,7 +13900,7 @@
       <c r="CO68" s="30"/>
       <c r="CP68" s="30"/>
     </row>
-    <row r="69" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="69" spans="27:94">
       <c r="AA69" s="29" t="s">
         <v>37</v>
       </c>
@@ -13892,7 +13972,7 @@
       <c r="CO69" s="30"/>
       <c r="CP69" s="30"/>
     </row>
-    <row r="70" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="70" spans="27:94">
       <c r="AA70" s="29" t="s">
         <v>38</v>
       </c>
@@ -13964,7 +14044,7 @@
       <c r="CO70" s="30"/>
       <c r="CP70" s="30"/>
     </row>
-    <row r="71" spans="27:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="27:94" ht="15" thickBot="1">
       <c r="AB71" s="23" t="s">
         <v>17</v>
       </c>
@@ -14031,8 +14111,8 @@
       <c r="CO71" s="39"/>
       <c r="CP71" s="40"/>
     </row>
-    <row r="73" spans="27:94" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="27:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="27:94" ht="15" thickBot="1"/>
+    <row r="74" spans="27:94" ht="15" thickBot="1">
       <c r="AA74" s="45" t="s">
         <v>46</v>
       </c>
@@ -14104,7 +14184,7 @@
       <c r="CO74" s="51"/>
       <c r="CP74" s="52"/>
     </row>
-    <row r="75" spans="27:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="27:94" ht="15" thickBot="1">
       <c r="AA75" s="1"/>
       <c r="AB75" s="5" t="s">
         <v>55</v>
@@ -14226,7 +14306,7 @@
       </c>
       <c r="CP75" s="44"/>
     </row>
-    <row r="76" spans="27:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="27:94" ht="15" thickBot="1">
       <c r="AA76" s="6" t="s">
         <v>0</v>
       </c>
@@ -14408,7 +14488,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="77" spans="27:94" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="27:94" ht="15" thickTop="1">
       <c r="AA77" s="48" t="s">
         <v>13</v>
       </c>
@@ -14490,7 +14570,7 @@
       <c r="CO77" s="19"/>
       <c r="CP77" s="20"/>
     </row>
-    <row r="78" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="78" spans="27:94">
       <c r="AA78" s="49"/>
       <c r="AB78" s="9" t="s">
         <v>11</v>
@@ -14562,7 +14642,7 @@
       <c r="CO78" s="15"/>
       <c r="CP78" s="16"/>
     </row>
-    <row r="79" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="79" spans="27:94">
       <c r="AA79" s="49"/>
       <c r="AB79" s="9" t="s">
         <v>12</v>
@@ -14634,7 +14714,7 @@
       <c r="CO79" s="15"/>
       <c r="CP79" s="16"/>
     </row>
-    <row r="80" spans="27:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="27:94" ht="15" thickBot="1">
       <c r="AA80" s="50"/>
       <c r="AB80" s="10" t="s">
         <v>14</v>
@@ -14706,8 +14786,8 @@
       <c r="CO80" s="21"/>
       <c r="CP80" s="22"/>
     </row>
-    <row r="82" spans="27:94" ht="16" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="27:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="27:94" ht="15" thickBot="1"/>
+    <row r="83" spans="27:94" ht="15" thickBot="1">
       <c r="AA83" s="45" t="s">
         <v>47</v>
       </c>
@@ -14779,7 +14859,7 @@
       <c r="CO83" s="46"/>
       <c r="CP83" s="47"/>
     </row>
-    <row r="84" spans="27:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="27:94" ht="15" thickBot="1">
       <c r="AA84" s="24"/>
       <c r="AB84" s="5" t="s">
         <v>55</v>
@@ -14901,7 +14981,7 @@
       </c>
       <c r="CP84" s="44"/>
     </row>
-    <row r="85" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="85" spans="27:94">
       <c r="AA85" s="25" t="s">
         <v>16</v>
       </c>
@@ -15083,7 +15163,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="86" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="86" spans="27:94">
       <c r="AA86" s="29" t="s">
         <v>24</v>
       </c>
@@ -15155,7 +15235,7 @@
       <c r="CO86" s="30"/>
       <c r="CP86" s="30"/>
     </row>
-    <row r="87" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="87" spans="27:94">
       <c r="AA87" s="29" t="s">
         <v>39</v>
       </c>
@@ -15227,7 +15307,7 @@
       <c r="CO87" s="30"/>
       <c r="CP87" s="30"/>
     </row>
-    <row r="88" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="88" spans="27:94">
       <c r="AA88" s="29" t="s">
         <v>20</v>
       </c>
@@ -15299,7 +15379,7 @@
       <c r="CO88" s="34"/>
       <c r="CP88" s="34"/>
     </row>
-    <row r="89" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="89" spans="27:94">
       <c r="AA89" s="29" t="s">
         <v>29</v>
       </c>
@@ -15371,7 +15451,7 @@
       <c r="CO89" s="34"/>
       <c r="CP89" s="34"/>
     </row>
-    <row r="90" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="90" spans="27:94">
       <c r="AA90" s="29" t="s">
         <v>25</v>
       </c>
@@ -15443,7 +15523,7 @@
       <c r="CO90" s="30"/>
       <c r="CP90" s="30"/>
     </row>
-    <row r="91" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="91" spans="27:94">
       <c r="AA91" s="29" t="s">
         <v>21</v>
       </c>
@@ -15515,7 +15595,7 @@
       <c r="CO91" s="30"/>
       <c r="CP91" s="30"/>
     </row>
-    <row r="92" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="92" spans="27:94">
       <c r="AA92" s="29" t="s">
         <v>30</v>
       </c>
@@ -15587,7 +15667,7 @@
       <c r="CO92" s="34"/>
       <c r="CP92" s="34"/>
     </row>
-    <row r="93" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="93" spans="27:94">
       <c r="AA93" s="29" t="s">
         <v>26</v>
       </c>
@@ -15659,7 +15739,7 @@
       <c r="CO93" s="30"/>
       <c r="CP93" s="30"/>
     </row>
-    <row r="94" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="94" spans="27:94">
       <c r="AA94" s="29" t="s">
         <v>22</v>
       </c>
@@ -15726,7 +15806,7 @@
       <c r="CO94" s="30"/>
       <c r="CP94" s="30"/>
     </row>
-    <row r="95" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="95" spans="27:94">
       <c r="AA95" s="29" t="s">
         <v>23</v>
       </c>
@@ -15798,7 +15878,7 @@
       <c r="CO95" s="30"/>
       <c r="CP95" s="30"/>
     </row>
-    <row r="96" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="96" spans="27:94">
       <c r="AA96" s="29" t="s">
         <v>31</v>
       </c>
@@ -15870,7 +15950,7 @@
       <c r="CO96" s="30"/>
       <c r="CP96" s="30"/>
     </row>
-    <row r="97" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="97" spans="27:94">
       <c r="AA97" s="29" t="s">
         <v>40</v>
       </c>
@@ -15942,7 +16022,7 @@
       <c r="CO97" s="30"/>
       <c r="CP97" s="30"/>
     </row>
-    <row r="98" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="98" spans="27:94">
       <c r="AA98" s="29" t="s">
         <v>27</v>
       </c>
@@ -16014,7 +16094,7 @@
       <c r="CO98" s="30"/>
       <c r="CP98" s="30"/>
     </row>
-    <row r="99" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="99" spans="27:94">
       <c r="AA99" s="29" t="s">
         <v>32</v>
       </c>
@@ -16086,7 +16166,7 @@
       <c r="CO99" s="30"/>
       <c r="CP99" s="30"/>
     </row>
-    <row r="100" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="100" spans="27:94">
       <c r="AA100" s="29" t="s">
         <v>28</v>
       </c>
@@ -16158,7 +16238,7 @@
       <c r="CO100" s="30"/>
       <c r="CP100" s="30"/>
     </row>
-    <row r="101" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="101" spans="27:94">
       <c r="AA101" s="29" t="s">
         <v>33</v>
       </c>
@@ -16230,7 +16310,7 @@
       <c r="CO101" s="30"/>
       <c r="CP101" s="30"/>
     </row>
-    <row r="102" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="102" spans="27:94">
       <c r="AA102" s="29" t="s">
         <v>34</v>
       </c>
@@ -16302,7 +16382,7 @@
       <c r="CO102" s="30"/>
       <c r="CP102" s="30"/>
     </row>
-    <row r="103" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="103" spans="27:94">
       <c r="AA103" s="29" t="s">
         <v>35</v>
       </c>
@@ -16374,7 +16454,7 @@
       <c r="CO103" s="30"/>
       <c r="CP103" s="30"/>
     </row>
-    <row r="104" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="104" spans="27:94">
       <c r="AA104" s="29" t="s">
         <v>36</v>
       </c>
@@ -16446,7 +16526,7 @@
       <c r="CO104" s="30"/>
       <c r="CP104" s="30"/>
     </row>
-    <row r="105" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="105" spans="27:94">
       <c r="AA105" s="29" t="s">
         <v>37</v>
       </c>
@@ -16518,7 +16598,7 @@
       <c r="CO105" s="30"/>
       <c r="CP105" s="30"/>
     </row>
-    <row r="106" spans="27:94" x14ac:dyDescent="0.2">
+    <row r="106" spans="27:94">
       <c r="AA106" s="29" t="s">
         <v>38</v>
       </c>
@@ -16590,7 +16670,7 @@
       <c r="CO106" s="30"/>
       <c r="CP106" s="30"/>
     </row>
-    <row r="107" spans="27:94" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="27:94" ht="15" thickBot="1">
       <c r="AB107" s="23" t="s">
         <v>17</v>
       </c>
@@ -16933,6 +17013,12 @@
     <mergeCell ref="BI107:BJ107"/>
     <mergeCell ref="BK107:BL107"/>
     <mergeCell ref="BM107:BN107"/>
+    <mergeCell ref="CO107:CP107"/>
+    <mergeCell ref="BS107:BT107"/>
+    <mergeCell ref="BU107:BV107"/>
+    <mergeCell ref="BW107:BX107"/>
+    <mergeCell ref="BY107:BZ107"/>
+    <mergeCell ref="CA107:CB107"/>
     <mergeCell ref="AQ107:AR107"/>
     <mergeCell ref="AS107:AT107"/>
     <mergeCell ref="AU107:AV107"/>
@@ -16942,12 +17028,6 @@
     <mergeCell ref="CI107:CJ107"/>
     <mergeCell ref="CK107:CL107"/>
     <mergeCell ref="CM107:CN107"/>
-    <mergeCell ref="CO107:CP107"/>
-    <mergeCell ref="BS107:BT107"/>
-    <mergeCell ref="BU107:BV107"/>
-    <mergeCell ref="BW107:BX107"/>
-    <mergeCell ref="BY107:BZ107"/>
-    <mergeCell ref="CA107:CB107"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>